<commit_message>
Sprint 4 - Duration Analytics
</commit_message>
<xml_diff>
--- a/exports/QuantLab_Report.xlsx
+++ b/exports/QuantLab_Report.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Monthly" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Weekly" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Weekday" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Duration" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -64086,4 +64087,407 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Duration Analytics</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Duration Bucket</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Trades</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Wins</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Losses</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Win %</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Gross Profit</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Gross Loss</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Net Profit</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Avg P&amp;L</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Best Trade</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Worst Trade</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Profit Factor</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0-15 min</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>121497.22</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-121497.22</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-2429.9444</v>
+      </c>
+      <c r="J4" t="n">
+        <v>-2102.78</v>
+      </c>
+      <c r="K4" t="n">
+        <v>-3189.55</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>15-30 min</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>29</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>29</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>74227.74000000001</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-74227.74000000001</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-2559.577241379311</v>
+      </c>
+      <c r="J5" t="n">
+        <v>-2079.53</v>
+      </c>
+      <c r="K5" t="n">
+        <v>-4116.87</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>30-60 min</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>36</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>36</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>87898.33</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-87898.33</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-2441.620277777778</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-2071.91</v>
+      </c>
+      <c r="K6" t="n">
+        <v>-4413.44</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1-2 hrs</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>33</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>33</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>78864.06999999999</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-78864.06999999999</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-2389.820303030303</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-2051.03</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-4177.73</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2-4 hrs</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>34</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>34</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>85762.44</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-85762.44</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-2522.424705882353</v>
+      </c>
+      <c r="J8" t="n">
+        <v>-2088.24</v>
+      </c>
+      <c r="K8" t="n">
+        <v>-5203.57</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>4-6 hrs</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>204</v>
+      </c>
+      <c r="C9" t="n">
+        <v>187</v>
+      </c>
+      <c r="D9" t="n">
+        <v>17</v>
+      </c>
+      <c r="E9" t="n">
+        <v>91.66666666666666</v>
+      </c>
+      <c r="F9" t="n">
+        <v>758695.64</v>
+      </c>
+      <c r="G9" t="n">
+        <v>30755.44</v>
+      </c>
+      <c r="H9" t="n">
+        <v>727940.2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3568.33431372549</v>
+      </c>
+      <c r="J9" t="n">
+        <v>15938.81</v>
+      </c>
+      <c r="K9" t="n">
+        <v>-3611.17</v>
+      </c>
+      <c r="L9" t="n">
+        <v>24.66866479556137</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>6+ hrs Same Day</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Overnight / Multi-day</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Sprint 5 - Streak Analytics
</commit_message>
<xml_diff>
--- a/exports/QuantLab_Report.xlsx
+++ b/exports/QuantLab_Report.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Weekly" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Weekday" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Duration" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Streak" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -64490,4 +64491,2926 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C229"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Streak Analytics</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Longest Winning Streak</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Longest Losing Streak</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Average Winning Streak</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Average Losing Streak</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1.86</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Total Winning Streaks</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Total Losing Streaks</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Current Streak Type</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Current Streak Length</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Largest Winning Streak P&amp;L</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>33423.18</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Largest Losing Streak P&amp;L</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>-18117.88</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Streak Type</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Length</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1284.97</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>-2326.06</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>4</v>
+      </c>
+      <c r="C18" t="n">
+        <v>5579.13</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" t="n">
+        <v>-2200.75</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="n">
+        <v>7312.38</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" t="n">
+        <v>-13807.33</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="n">
+        <v>4545.86</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="n">
+        <v>-2166.68</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2644.59</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>-2223.47</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" t="n">
+        <v>6860.96</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="n">
+        <v>-4554.34</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" t="n">
+        <v>7082.06</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" t="n">
+        <v>-2112.32</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>2</v>
+      </c>
+      <c r="C30" t="n">
+        <v>6306.16</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" t="n">
+        <v>-5177.03</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="n">
+        <v>3535.55</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>-2107.22</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" t="n">
+        <v>6945.01</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>-2083.62</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>2835.69</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>-2427.94</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>3590.03</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>2</v>
+      </c>
+      <c r="C39" t="n">
+        <v>-4264.32</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>3312.17</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" t="n">
+        <v>-4227.29</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>5</v>
+      </c>
+      <c r="C42" t="n">
+        <v>6411.46</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>-2500.66</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>556.11</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>-2803.27</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>6987.69</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="n">
+        <v>-4939.78</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>9730.5</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>4</v>
+      </c>
+      <c r="C49" t="n">
+        <v>-10063.71</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" t="n">
+        <v>6730.59</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="n">
+        <v>-4490.7</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2</v>
+      </c>
+      <c r="C52" t="n">
+        <v>9027.41</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>6</v>
+      </c>
+      <c r="C53" t="n">
+        <v>-13995.08</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="n">
+        <v>5165.94</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" t="n">
+        <v>-2094.84</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>4</v>
+      </c>
+      <c r="C56" t="n">
+        <v>10388.91</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" t="n">
+        <v>-2388.9</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>2</v>
+      </c>
+      <c r="C58" t="n">
+        <v>7584.49</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>3</v>
+      </c>
+      <c r="C59" t="n">
+        <v>-6625.04</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" t="n">
+        <v>2998.68</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>2</v>
+      </c>
+      <c r="C61" t="n">
+        <v>-4713.68</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>2</v>
+      </c>
+      <c r="C62" t="n">
+        <v>8423.5</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C63" t="n">
+        <v>-2135.67</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" t="n">
+        <v>3237.93</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>3</v>
+      </c>
+      <c r="C65" t="n">
+        <v>-6757.52</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" t="n">
+        <v>5847.33</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" t="n">
+        <v>-2245.78</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>2</v>
+      </c>
+      <c r="C68" t="n">
+        <v>6492.44</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" t="n">
+        <v>-2694.1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>3</v>
+      </c>
+      <c r="C70" t="n">
+        <v>9212.459999999999</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" t="n">
+        <v>-2284.78</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>3</v>
+      </c>
+      <c r="C72" t="n">
+        <v>18609.53</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>1</v>
+      </c>
+      <c r="C73" t="n">
+        <v>-2218.5</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>1</v>
+      </c>
+      <c r="C74" t="n">
+        <v>3278.76</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>2</v>
+      </c>
+      <c r="C75" t="n">
+        <v>-4582.27</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>4</v>
+      </c>
+      <c r="C76" t="n">
+        <v>13776.12</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>5</v>
+      </c>
+      <c r="C77" t="n">
+        <v>-9717.639999999999</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>2</v>
+      </c>
+      <c r="C78" t="n">
+        <v>6304.2</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>5</v>
+      </c>
+      <c r="C79" t="n">
+        <v>-10608.35</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>2</v>
+      </c>
+      <c r="C80" t="n">
+        <v>6763.97</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>4</v>
+      </c>
+      <c r="C81" t="n">
+        <v>-8843.950000000001</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>2</v>
+      </c>
+      <c r="C82" t="n">
+        <v>7315.35</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>1</v>
+      </c>
+      <c r="C83" t="n">
+        <v>-2120.35</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>5</v>
+      </c>
+      <c r="C84" t="n">
+        <v>28254.05</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>3</v>
+      </c>
+      <c r="C85" t="n">
+        <v>-6864.96</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>6</v>
+      </c>
+      <c r="C86" t="n">
+        <v>18489.37</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>1</v>
+      </c>
+      <c r="C87" t="n">
+        <v>-2963.19</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>1</v>
+      </c>
+      <c r="C88" t="n">
+        <v>5602.61</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>2</v>
+      </c>
+      <c r="C89" t="n">
+        <v>-4778.15</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>2</v>
+      </c>
+      <c r="C90" t="n">
+        <v>18660.85</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>3</v>
+      </c>
+      <c r="C91" t="n">
+        <v>-7000.61</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>1</v>
+      </c>
+      <c r="C92" t="n">
+        <v>4253.15</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>1</v>
+      </c>
+      <c r="C93" t="n">
+        <v>-2301.75</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>1</v>
+      </c>
+      <c r="C94" t="n">
+        <v>4818.6</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>3</v>
+      </c>
+      <c r="C95" t="n">
+        <v>-8610.66</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>2</v>
+      </c>
+      <c r="C96" t="n">
+        <v>11408.43</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>3</v>
+      </c>
+      <c r="C97" t="n">
+        <v>-9719.74</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>1</v>
+      </c>
+      <c r="C98" t="n">
+        <v>9143.129999999999</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>1</v>
+      </c>
+      <c r="C99" t="n">
+        <v>-2465.27</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>2</v>
+      </c>
+      <c r="C100" t="n">
+        <v>7235.78</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>3</v>
+      </c>
+      <c r="C101" t="n">
+        <v>-6815.42</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>2</v>
+      </c>
+      <c r="C102" t="n">
+        <v>9121.49</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>1</v>
+      </c>
+      <c r="C103" t="n">
+        <v>-2124.56</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>1</v>
+      </c>
+      <c r="C104" t="n">
+        <v>6409.59</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>1</v>
+      </c>
+      <c r="C105" t="n">
+        <v>-2313.29</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>4</v>
+      </c>
+      <c r="C106" t="n">
+        <v>22767.38</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>1</v>
+      </c>
+      <c r="C107" t="n">
+        <v>-2149.5</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>1</v>
+      </c>
+      <c r="C108" t="n">
+        <v>3986.47</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>1</v>
+      </c>
+      <c r="C109" t="n">
+        <v>-2320.34</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>1</v>
+      </c>
+      <c r="C110" t="n">
+        <v>2690.94</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>1</v>
+      </c>
+      <c r="C111" t="n">
+        <v>-2242.84</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>2</v>
+      </c>
+      <c r="C112" t="n">
+        <v>5889.66</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>1</v>
+      </c>
+      <c r="C113" t="n">
+        <v>-2235.07</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>1</v>
+      </c>
+      <c r="C114" t="n">
+        <v>2710.53</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>1</v>
+      </c>
+      <c r="C115" t="n">
+        <v>-2161.88</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>1</v>
+      </c>
+      <c r="C116" t="n">
+        <v>4917.3</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>2</v>
+      </c>
+      <c r="C117" t="n">
+        <v>-5145.55</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>2</v>
+      </c>
+      <c r="C118" t="n">
+        <v>10047.97</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>1</v>
+      </c>
+      <c r="C119" t="n">
+        <v>-2797.83</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>2</v>
+      </c>
+      <c r="C120" t="n">
+        <v>10103.73</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>1</v>
+      </c>
+      <c r="C121" t="n">
+        <v>-2162.83</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>1</v>
+      </c>
+      <c r="C122" t="n">
+        <v>3898.37</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>1</v>
+      </c>
+      <c r="C123" t="n">
+        <v>-2298.45</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>2</v>
+      </c>
+      <c r="C124" t="n">
+        <v>9121.08</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>4</v>
+      </c>
+      <c r="C125" t="n">
+        <v>-8798.51</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>2</v>
+      </c>
+      <c r="C126" t="n">
+        <v>4392.03</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>3</v>
+      </c>
+      <c r="C127" t="n">
+        <v>-6330.35</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>1</v>
+      </c>
+      <c r="C128" t="n">
+        <v>4163.51</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>1</v>
+      </c>
+      <c r="C129" t="n">
+        <v>-842.38</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>2</v>
+      </c>
+      <c r="C130" t="n">
+        <v>7861.13</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>1</v>
+      </c>
+      <c r="C131" t="n">
+        <v>-2259.48</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>1</v>
+      </c>
+      <c r="C132" t="n">
+        <v>4074.46</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>4</v>
+      </c>
+      <c r="C133" t="n">
+        <v>-9089.6</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>1</v>
+      </c>
+      <c r="C134" t="n">
+        <v>5721.97</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>1</v>
+      </c>
+      <c r="C135" t="n">
+        <v>-2102.78</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>3</v>
+      </c>
+      <c r="C136" t="n">
+        <v>12471.37</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>2</v>
+      </c>
+      <c r="C137" t="n">
+        <v>-4584.32</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>2</v>
+      </c>
+      <c r="C138" t="n">
+        <v>7423.68</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>1</v>
+      </c>
+      <c r="C139" t="n">
+        <v>-2217.52</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>2</v>
+      </c>
+      <c r="C140" t="n">
+        <v>3639.18</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>1</v>
+      </c>
+      <c r="C141" t="n">
+        <v>-2247.9</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>3</v>
+      </c>
+      <c r="C142" t="n">
+        <v>8677.190000000001</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>1</v>
+      </c>
+      <c r="C143" t="n">
+        <v>-4177.73</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>3</v>
+      </c>
+      <c r="C144" t="n">
+        <v>4260.68</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>2</v>
+      </c>
+      <c r="C145" t="n">
+        <v>-5901.57</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>1</v>
+      </c>
+      <c r="C146" t="n">
+        <v>3485.37</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>1</v>
+      </c>
+      <c r="C147" t="n">
+        <v>-2208.07</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>1</v>
+      </c>
+      <c r="C148" t="n">
+        <v>3501.19</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>1</v>
+      </c>
+      <c r="C149" t="n">
+        <v>-2295.23</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>1</v>
+      </c>
+      <c r="C150" t="n">
+        <v>6125.24</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>1</v>
+      </c>
+      <c r="C151" t="n">
+        <v>-3691.22</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>1</v>
+      </c>
+      <c r="C152" t="n">
+        <v>7084.24</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>3</v>
+      </c>
+      <c r="C153" t="n">
+        <v>-7658.64</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>1</v>
+      </c>
+      <c r="C154" t="n">
+        <v>3648.56</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>8</v>
+      </c>
+      <c r="C155" t="n">
+        <v>-18117.88</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>1</v>
+      </c>
+      <c r="C156" t="n">
+        <v>8598.83</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>2</v>
+      </c>
+      <c r="C157" t="n">
+        <v>-4990.32</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>1</v>
+      </c>
+      <c r="C158" t="n">
+        <v>7412.91</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>1</v>
+      </c>
+      <c r="C159" t="n">
+        <v>-4413.44</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>1</v>
+      </c>
+      <c r="C160" t="n">
+        <v>4030.59</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>2</v>
+      </c>
+      <c r="C161" t="n">
+        <v>-4886.63</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>2</v>
+      </c>
+      <c r="C162" t="n">
+        <v>5908.56</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>2</v>
+      </c>
+      <c r="C163" t="n">
+        <v>-4699.89</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>1</v>
+      </c>
+      <c r="C164" t="n">
+        <v>4916.15</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>1</v>
+      </c>
+      <c r="C165" t="n">
+        <v>-3062.9</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>2</v>
+      </c>
+      <c r="C166" t="n">
+        <v>5465.83</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>1</v>
+      </c>
+      <c r="C167" t="n">
+        <v>-3032.83</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>1</v>
+      </c>
+      <c r="C168" t="n">
+        <v>4446.5</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>1</v>
+      </c>
+      <c r="C169" t="n">
+        <v>-3611.17</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>1</v>
+      </c>
+      <c r="C170" t="n">
+        <v>4790.83</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>1</v>
+      </c>
+      <c r="C171" t="n">
+        <v>-3325.79</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>1</v>
+      </c>
+      <c r="C172" t="n">
+        <v>10830.66</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>1</v>
+      </c>
+      <c r="C173" t="n">
+        <v>-2173.05</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>1</v>
+      </c>
+      <c r="C174" t="n">
+        <v>4919.38</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>1</v>
+      </c>
+      <c r="C175" t="n">
+        <v>-2285.12</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>2</v>
+      </c>
+      <c r="C176" t="n">
+        <v>10395.63</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>4</v>
+      </c>
+      <c r="C177" t="n">
+        <v>-9088.92</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>3</v>
+      </c>
+      <c r="C178" t="n">
+        <v>9652.24</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>2</v>
+      </c>
+      <c r="C179" t="n">
+        <v>-4593.39</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>1</v>
+      </c>
+      <c r="C180" t="n">
+        <v>550.84</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>2</v>
+      </c>
+      <c r="C181" t="n">
+        <v>-6654.84</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>1</v>
+      </c>
+      <c r="C182" t="n">
+        <v>6200.45</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>1</v>
+      </c>
+      <c r="C183" t="n">
+        <v>-2306.62</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>2</v>
+      </c>
+      <c r="C184" t="n">
+        <v>5677.34</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>5</v>
+      </c>
+      <c r="C185" t="n">
+        <v>-12030.77</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>1</v>
+      </c>
+      <c r="C186" t="n">
+        <v>5959.62</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>1</v>
+      </c>
+      <c r="C187" t="n">
+        <v>-2307.06</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>1</v>
+      </c>
+      <c r="C188" t="n">
+        <v>2755.14</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>1</v>
+      </c>
+      <c r="C189" t="n">
+        <v>-2216.5</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>1</v>
+      </c>
+      <c r="C190" t="n">
+        <v>2917.8</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>1</v>
+      </c>
+      <c r="C191" t="n">
+        <v>-2504.01</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>1</v>
+      </c>
+      <c r="C192" t="n">
+        <v>3348.48</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>2</v>
+      </c>
+      <c r="C193" t="n">
+        <v>-6147.41</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>2</v>
+      </c>
+      <c r="C194" t="n">
+        <v>10789.27</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>2</v>
+      </c>
+      <c r="C195" t="n">
+        <v>-4910.33</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>3</v>
+      </c>
+      <c r="C196" t="n">
+        <v>12937.69</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>2</v>
+      </c>
+      <c r="C197" t="n">
+        <v>-4609.28</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>1</v>
+      </c>
+      <c r="C198" t="n">
+        <v>2926.09</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>3</v>
+      </c>
+      <c r="C199" t="n">
+        <v>-6704.73</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>1</v>
+      </c>
+      <c r="C200" t="n">
+        <v>1930.35</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>2</v>
+      </c>
+      <c r="C201" t="n">
+        <v>-5211.96</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>1</v>
+      </c>
+      <c r="C202" t="n">
+        <v>4511.05</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>1</v>
+      </c>
+      <c r="C203" t="n">
+        <v>-2111.64</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>1</v>
+      </c>
+      <c r="C204" t="n">
+        <v>5126.47</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>1</v>
+      </c>
+      <c r="C205" t="n">
+        <v>-2294.83</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>2</v>
+      </c>
+      <c r="C206" t="n">
+        <v>12962.46</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>1</v>
+      </c>
+      <c r="C207" t="n">
+        <v>-2896.89</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>1</v>
+      </c>
+      <c r="C208" t="n">
+        <v>4656.18</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>1</v>
+      </c>
+      <c r="C209" t="n">
+        <v>-2445.9</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>1</v>
+      </c>
+      <c r="C210" t="n">
+        <v>4826.9</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>1</v>
+      </c>
+      <c r="C211" t="n">
+        <v>-3079.29</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>1</v>
+      </c>
+      <c r="C212" t="n">
+        <v>4173.47</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>1</v>
+      </c>
+      <c r="C213" t="n">
+        <v>-2544.38</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>1</v>
+      </c>
+      <c r="C214" t="n">
+        <v>3056.67</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>2</v>
+      </c>
+      <c r="C215" t="n">
+        <v>-4772.52</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>2</v>
+      </c>
+      <c r="C216" t="n">
+        <v>10882.44</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>1</v>
+      </c>
+      <c r="C217" t="n">
+        <v>-2349.34</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>1</v>
+      </c>
+      <c r="C218" t="n">
+        <v>4412.64</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>2</v>
+      </c>
+      <c r="C219" t="n">
+        <v>-4935.27</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>1</v>
+      </c>
+      <c r="C220" t="n">
+        <v>8159.55</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>3</v>
+      </c>
+      <c r="C221" t="n">
+        <v>-9096.17</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>1</v>
+      </c>
+      <c r="C222" t="n">
+        <v>15938.81</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>3</v>
+      </c>
+      <c r="C223" t="n">
+        <v>-8998</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>5</v>
+      </c>
+      <c r="C224" t="n">
+        <v>33423.18</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
+        <v>1</v>
+      </c>
+      <c r="C225" t="n">
+        <v>-2340.41</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>1</v>
+      </c>
+      <c r="C226" t="n">
+        <v>1261.28</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>1</v>
+      </c>
+      <c r="C227" t="n">
+        <v>-2596.36</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>1</v>
+      </c>
+      <c r="C228" t="n">
+        <v>5205.15</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>1</v>
+      </c>
+      <c r="C229" t="n">
+        <v>-2279.27</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Documentation Sprint - Phase 1 Architecture
</commit_message>
<xml_diff>
--- a/exports/QuantLab_Report.xlsx
+++ b/exports/QuantLab_Report.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Duration" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Streak" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Calendar" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Risk" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17241,6 +17242,137 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Risk Analytics</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Standard Deviation</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3617.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Downside Deviation</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>583.2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Sharpe Ratio</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Sortino Ratio</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1.242</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Calmar Ratio</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>16.167</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Ulcer Index</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.539</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Recovery Factor</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>12.64</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Value at Risk (95%)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>-3062.9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Conditional VaR (95%)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>-3611.34</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Kelly %</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>17.86</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Half Kelly %</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>8.93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>